<commit_message>
Prepare purchase request system 2.0 for Vercel
</commit_message>
<xml_diff>
--- a/purchase_request_backend_template.xlsx
+++ b/purchase_request_backend_template.xlsx
@@ -7,11 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Requests" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Items" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Approvals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Users" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="請購主表" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="品項明細" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="簽核紀錄" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用者權限" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系統設定" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -157,102 +157,100 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="RequestsTable" displayName="RequestsTable" ref="A1:X2" headerRowCount="1">
-  <autoFilter ref="A1:X2"/>
-  <tableColumns count="24">
-    <tableColumn id="1" name="request_id"/>
-    <tableColumn id="2" name="created_at"/>
-    <tableColumn id="3" name="updated_at"/>
-    <tableColumn id="4" name="employee_id"/>
-    <tableColumn id="5" name="employee_email"/>
-    <tableColumn id="6" name="applicant_name"/>
-    <tableColumn id="7" name="department_code"/>
-    <tableColumn id="8" name="request_type"/>
-    <tableColumn id="9" name="apply_date"/>
-    <tableColumn id="10" name="need_date"/>
-    <tableColumn id="11" name="vendor_name"/>
-    <tableColumn id="12" name="vendor_tax_id"/>
-    <tableColumn id="13" name="tax_type"/>
-    <tableColumn id="14" name="total_amount"/>
-    <tableColumn id="15" name="approval_status"/>
-    <tableColumn id="16" name="current_step"/>
-    <tableColumn id="17" name="categories"/>
-    <tableColumn id="18" name="attachments"/>
-    <tableColumn id="19" name="purpose"/>
-    <tableColumn id="20" name="acceptance_note"/>
-    <tableColumn id="21" name="photo_count"/>
-    <tableColumn id="22" name="signature_status"/>
-    <tableColumn id="23" name="notion_page_url"/>
-    <tableColumn id="24" name="raw_json"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:W2" headerRowCount="1">
+  <autoFilter ref="A1:W2"/>
+  <tableColumns count="23">
+    <tableColumn id="1" name="單號"/>
+    <tableColumn id="2" name="建立時間"/>
+    <tableColumn id="3" name="更新時間"/>
+    <tableColumn id="4" name="員工編號"/>
+    <tableColumn id="5" name="公司信箱"/>
+    <tableColumn id="6" name="申請人"/>
+    <tableColumn id="7" name="部門代號"/>
+    <tableColumn id="8" name="申請類型"/>
+    <tableColumn id="9" name="申請日期"/>
+    <tableColumn id="10" name="須用日期"/>
+    <tableColumn id="11" name="廠商名稱"/>
+    <tableColumn id="12" name="統一編號"/>
+    <tableColumn id="13" name="稅別"/>
+    <tableColumn id="14" name="合計金額"/>
+    <tableColumn id="15" name="簽核狀態"/>
+    <tableColumn id="16" name="目前關卡"/>
+    <tableColumn id="17" name="類別"/>
+    <tableColumn id="18" name="檢附資料"/>
+    <tableColumn id="19" name="用途說明"/>
+    <tableColumn id="20" name="驗收/其他說明"/>
+    <tableColumn id="21" name="照片數"/>
+    <tableColumn id="22" name="簽名狀態"/>
+    <tableColumn id="23" name="原始資料"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ItemsTable" displayName="ItemsTable" ref="A1:K2" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:K2" headerRowCount="1">
   <autoFilter ref="A1:K2"/>
   <tableColumns count="11">
-    <tableColumn id="1" name="request_id"/>
-    <tableColumn id="2" name="line_no"/>
-    <tableColumn id="3" name="item_name"/>
-    <tableColumn id="4" name="spec"/>
-    <tableColumn id="5" name="item_code"/>
-    <tableColumn id="6" name="unit"/>
-    <tableColumn id="7" name="qty"/>
-    <tableColumn id="8" name="approved_qty"/>
-    <tableColumn id="9" name="unit_price"/>
-    <tableColumn id="10" name="amount"/>
-    <tableColumn id="11" name="note"/>
+    <tableColumn id="1" name="單號"/>
+    <tableColumn id="2" name="項次"/>
+    <tableColumn id="3" name="品項名稱"/>
+    <tableColumn id="4" name="規格"/>
+    <tableColumn id="5" name="品項編號"/>
+    <tableColumn id="6" name="單位"/>
+    <tableColumn id="7" name="申購數量"/>
+    <tableColumn id="8" name="核准數量"/>
+    <tableColumn id="9" name="單價"/>
+    <tableColumn id="10" name="金額"/>
+    <tableColumn id="11" name="備註"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="ApprovalsTable" displayName="ApprovalsTable" ref="A1:J2" headerRowCount="1">
-  <autoFilter ref="A1:J2"/>
-  <tableColumns count="10">
-    <tableColumn id="1" name="request_id"/>
-    <tableColumn id="2" name="action_at"/>
-    <tableColumn id="3" name="step"/>
-    <tableColumn id="4" name="action"/>
-    <tableColumn id="5" name="actor_employee_id"/>
-    <tableColumn id="6" name="actor_name"/>
-    <tableColumn id="7" name="actor_email"/>
-    <tableColumn id="8" name="note"/>
-    <tableColumn id="9" name="notify_email"/>
-    <tableColumn id="10" name="notion_page_url"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="Table3" displayName="Table3" ref="A1:I2" headerRowCount="1">
+  <autoFilter ref="A1:I2"/>
+  <tableColumns count="9">
+    <tableColumn id="1" name="單號"/>
+    <tableColumn id="2" name="動作時間"/>
+    <tableColumn id="3" name="關卡"/>
+    <tableColumn id="4" name="動作"/>
+    <tableColumn id="5" name="簽核人工號"/>
+    <tableColumn id="6" name="簽核人"/>
+    <tableColumn id="7" name="簽核人信箱"/>
+    <tableColumn id="8" name="說明"/>
+    <tableColumn id="9" name="通知信箱"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="UsersTable" displayName="UsersTable" ref="A1:I4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:I4" headerRowCount="1">
   <autoFilter ref="A1:I4"/>
   <tableColumns count="9">
-    <tableColumn id="1" name="employee_id"/>
-    <tableColumn id="2" name="name"/>
-    <tableColumn id="3" name="email"/>
-    <tableColumn id="4" name="department_code"/>
-    <tableColumn id="5" name="role"/>
-    <tableColumn id="6" name="is_active"/>
-    <tableColumn id="7" name="created_at"/>
-    <tableColumn id="8" name="updated_at"/>
-    <tableColumn id="9" name="note"/>
+    <tableColumn id="1" name="員工編號"/>
+    <tableColumn id="2" name="姓名"/>
+    <tableColumn id="3" name="公司信箱"/>
+    <tableColumn id="4" name="部門代號"/>
+    <tableColumn id="5" name="權限"/>
+    <tableColumn id="6" name="啟用"/>
+    <tableColumn id="7" name="建立時間"/>
+    <tableColumn id="8" name="更新時間"/>
+    <tableColumn id="9" name="備註"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="SettingsTable" displayName="SettingsTable" ref="A1:C4" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="Table5" displayName="Table5" ref="A1:C4" headerRowCount="1">
   <autoFilter ref="A1:C4"/>
   <tableColumns count="3">
-    <tableColumn id="1" name="setting_key"/>
-    <tableColumn id="2" name="setting_value"/>
-    <tableColumn id="3" name="description"/>
+    <tableColumn id="1" name="設定項目"/>
+    <tableColumn id="2" name="設定值"/>
+    <tableColumn id="3" name="說明"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -547,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X2"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -572,129 +570,123 @@
     <col width="30" customWidth="1" min="20" max="20"/>
     <col width="16" customWidth="1" min="21" max="21"/>
     <col width="16" customWidth="1" min="22" max="22"/>
-    <col width="16" customWidth="1" min="23" max="23"/>
-    <col width="36" customWidth="1" min="24" max="24"/>
+    <col width="36" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>request_id</t>
+          <t>單號</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>建立時間</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>更新時間</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>employee_id</t>
+          <t>員工編號</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>employee_email</t>
+          <t>公司信箱</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>applicant_name</t>
+          <t>申請人</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>department_code</t>
+          <t>部門代號</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>request_type</t>
+          <t>申請類型</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>apply_date</t>
+          <t>申請日期</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>need_date</t>
+          <t>須用日期</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>vendor_name</t>
+          <t>廠商名稱</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>vendor_tax_id</t>
+          <t>統一編號</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>tax_type</t>
+          <t>稅別</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>total_amount</t>
+          <t>合計金額</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>approval_status</t>
+          <t>簽核狀態</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>current_step</t>
+          <t>目前關卡</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>categories</t>
+          <t>類別</t>
         </is>
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
-          <t>attachments</t>
+          <t>檢附資料</t>
         </is>
       </c>
       <c r="S1" s="1" t="inlineStr">
         <is>
-          <t>purpose</t>
+          <t>用途說明</t>
         </is>
       </c>
       <c r="T1" s="1" t="inlineStr">
         <is>
-          <t>acceptance_note</t>
+          <t>驗收/其他說明</t>
         </is>
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>photo_count</t>
+          <t>照片數</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>signature_status</t>
+          <t>簽名狀態</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>notion_page_url</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>raw_json</t>
+          <t>原始資料</t>
         </is>
       </c>
     </row>
@@ -774,7 +766,7 @@
       </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>unitManager</t>
+          <t>單位主管</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -801,8 +793,7 @@
           <t>已簽名</t>
         </is>
       </c>
-      <c r="W2" s="2" t="inlineStr"/>
-      <c r="X2" s="2" t="inlineStr">
+      <c r="W2" s="2" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
@@ -849,57 +840,57 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>request_id</t>
+          <t>單號</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>line_no</t>
+          <t>項次</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>item_name</t>
+          <t>品項名稱</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>spec</t>
+          <t>規格</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>item_code</t>
+          <t>品項編號</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>unit</t>
+          <t>單位</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>qty</t>
+          <t>申購數量</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>approved_qty</t>
+          <t>核准數量</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>unit_price</t>
+          <t>單價</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>amount</t>
+          <t>金額</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
@@ -959,7 +950,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -969,60 +960,54 @@
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>request_id</t>
+          <t>單號</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>action_at</t>
+          <t>動作時間</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>step</t>
+          <t>關卡</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>action</t>
+          <t>動作</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>actor_employee_id</t>
+          <t>簽核人工號</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>actor_name</t>
+          <t>簽核人</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>actor_email</t>
+          <t>簽核人信箱</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>說明</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>notify_email</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>notion_page_url</t>
+          <t>通知信箱</t>
         </is>
       </c>
     </row>
@@ -1039,12 +1024,12 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>applicant</t>
+          <t>申請人</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>signed</t>
+          <t>已簽名</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -1072,7 +1057,6 @@
           <t>admin@example.com</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1093,7 +1077,7 @@
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
@@ -1105,47 +1089,47 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>employee_id</t>
+          <t>員工編號</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>姓名</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>email</t>
+          <t>公司信箱</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>department_code</t>
+          <t>部門代號</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>權限</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>is_active</t>
+          <t>啟用</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>created_at</t>
+          <t>建立時間</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>updated_at</t>
+          <t>更新時間</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>備註</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1152,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>admin</t>
+          <t>最高權限</t>
         </is>
       </c>
       <c r="F2" s="2" t="b">
@@ -1205,7 +1189,7 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>unitManager</t>
+          <t>單位主管</t>
         </is>
       </c>
       <c r="F3" s="3" t="b">
@@ -1238,7 +1222,7 @@
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>generalManager</t>
+          <t>總經理</t>
         </is>
       </c>
       <c r="F4" s="3" t="b">
@@ -1255,7 +1239,7 @@
   </sheetData>
   <dataValidations count="2">
     <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"user,unitManager,generalManager,admin"</formula1>
+      <formula1>"一般使用者,單位主管,總經理,最高權限"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"TRUE,FALSE"</formula1>
@@ -1285,24 +1269,24 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>setting_key</t>
+          <t>設定項目</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>setting_value</t>
+          <t>設定值</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>description</t>
+          <t>說明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>edit_limit_hours</t>
+          <t>可修改時限小時</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -1319,7 +1303,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>default_admin_employee_id</t>
+          <t>預設最高權限員工編號</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -1336,7 +1320,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>sheet_version</t>
+          <t>資料表版本</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">

</xml_diff>

<commit_message>
Build secure backend and approval admin
</commit_message>
<xml_diff>
--- a/purchase_request_backend_template.xlsx
+++ b/purchase_request_backend_template.xlsx
@@ -227,9 +227,9 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:I4" headerRowCount="1">
-  <autoFilter ref="A1:I4"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="Table4" displayName="Table4" ref="A1:J4" headerRowCount="1">
+  <autoFilter ref="A1:J4"/>
+  <tableColumns count="10">
     <tableColumn id="1" name="員工編號"/>
     <tableColumn id="2" name="姓名"/>
     <tableColumn id="3" name="公司信箱"/>
@@ -239,6 +239,7 @@
     <tableColumn id="7" name="建立時間"/>
     <tableColumn id="8" name="更新時間"/>
     <tableColumn id="9" name="備註"/>
+    <tableColumn id="10" name="密碼雜湊"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1072,7 +1073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1084,6 +1085,7 @@
     <col width="24" customWidth="1" min="7" max="7"/>
     <col width="24" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1132,6 +1134,11 @@
           <t>備註</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>密碼雜湊</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1169,6 +1176,7 @@
           <t>最高權限</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -1202,6 +1210,7 @@
       </c>
       <c r="H3" s="3" t="inlineStr"/>
       <c r="I3" s="3" t="inlineStr"/>
+      <c r="J3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1235,6 +1244,7 @@
       </c>
       <c r="H4" s="3" t="inlineStr"/>
       <c r="I4" s="3" t="inlineStr"/>
+      <c r="J4" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>